<commit_message>
some results changed about CEDIS
</commit_message>
<xml_diff>
--- a/CivisResults/CEDIS/4Objectives/Without Elec Car Introduction/Results_CEDIS 4 Objectives.xlsx
+++ b/CivisResults/CEDIS/4Objectives/Without Elec Car Introduction/Results_CEDIS 4 Objectives.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10995" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="4" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="49">
   <si>
     <t>Cost</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>AnnualHPheat</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
   </si>
 </sst>
 </file>
@@ -313,9 +319,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -326,6 +329,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -621,6 +627,928 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'15BestESD'!$AD$5:$AD$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>0.69</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.66</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.65</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.63</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.61</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.61</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.61</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.61</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.61</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'15BestESD'!$AE$5:$AE$19</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>0.40056622541893</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.40599892876272098</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="General">
+                  <c:v>0.406764098247761</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.41204376769454398</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.415104445634708</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.41625219986226902</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.41678781850179802</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.41709388629581401</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="General">
+                  <c:v>0.417246920192822</c:v>
+                </c:pt>
+                <c:pt idx="9" formatCode="General">
+                  <c:v>0.420613665927002</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.42145535236054699</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.42176142015456403</c:v>
+                </c:pt>
+                <c:pt idx="12" formatCode="General">
+                  <c:v>0.42260310658810901</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.42267962353661298</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="General">
+                  <c:v>0.42306220827913299</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="409415328"/>
+        <c:axId val="409416896"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="409415328"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="it-IT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="409416896"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="409416896"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="it-IT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="409415328"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="it-IT"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -688,7 +1616,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>These solutions are best 15 solutions in terms of annual cost (15% increase of current cost). 200 Solutions are sorted  by annual cost, co2 emission. LFC and ESD.</a:t>
+            <a:t>These solutions are best 15 solutions in terms of annual cost (15% increase of current cost). 200 Solutions are sorted  by annual cost, co2 emission, LFC and ESD.</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="it-IT" sz="1100" baseline="0">
@@ -708,6 +1636,41 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>519112</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>214312</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1013,74 +1976,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1170,25 +2133,25 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="AF3" s="12" t="s">
+      <c r="AF3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AG3" s="13" t="s">
+      <c r="AG3" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="AH3" s="13" t="s">
+      <c r="AH3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="AI3" s="13" t="s">
+      <c r="AI3" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="AJ3" s="13" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1280,13 +2243,13 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-      <c r="AI4" s="13"/>
-      <c r="AJ4" s="13"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
+      <c r="AF4" s="16"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="12"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
@@ -23431,6 +24394,11 @@
     <sortCondition ref="AE6:AE205"/>
   </sortState>
   <mergeCells count="15">
+    <mergeCell ref="AF3:AF4"/>
+    <mergeCell ref="AG3:AG4"/>
+    <mergeCell ref="AH3:AH4"/>
+    <mergeCell ref="AI3:AI4"/>
+    <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="J2:N2"/>
@@ -23441,11 +24409,6 @@
     <mergeCell ref="Q1:S2"/>
     <mergeCell ref="AB2:AE2"/>
     <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AF3:AF4"/>
-    <mergeCell ref="AG3:AG4"/>
-    <mergeCell ref="AH3:AH4"/>
-    <mergeCell ref="AI3:AI4"/>
-    <mergeCell ref="AJ3:AJ4"/>
   </mergeCells>
   <conditionalFormatting sqref="AC6:AC165">
     <cfRule type="cellIs" dxfId="26" priority="3" operator="lessThan">
@@ -23469,78 +24432,78 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -23630,25 +24593,25 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="AF3" s="12" t="s">
+      <c r="AF3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AG3" s="13" t="s">
+      <c r="AG3" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="AH3" s="13" t="s">
+      <c r="AH3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="AI3" s="13" t="s">
+      <c r="AI3" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="AJ3" s="13" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>46</v>
       </c>
     </row>
@@ -23740,13 +24703,13 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-      <c r="AI4" s="13"/>
-      <c r="AJ4" s="13"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
+      <c r="AF4" s="16"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="12"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -25398,8 +26361,56 @@
         <v>27.49</v>
       </c>
     </row>
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB21">
+        <f>MIN(AB5:AB19)</f>
+        <v>15.933</v>
+      </c>
+      <c r="AC21">
+        <f>MIN(AC5:AC19)</f>
+        <v>14100</v>
+      </c>
+      <c r="AD21">
+        <f>MIN(AD5:AD19)</f>
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="AE21">
+        <f>MIN(AE5:AE19)</f>
+        <v>0.42145535236054699</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA22" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <f>MAX(AB5:AB19)</f>
+        <v>16.478000000000002</v>
+      </c>
+      <c r="AC22">
+        <f>MAX(AC5:AC19)</f>
+        <v>14391</v>
+      </c>
+      <c r="AD22">
+        <f>MAX(AD5:AD19)</f>
+        <v>0.61</v>
+      </c>
+      <c r="AE22">
+        <f>MAX(AE5:AE19)</f>
+        <v>0.43683525900987002</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:N1"/>
+    <mergeCell ref="O1:P2"/>
+    <mergeCell ref="Q1:S2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="J2:N2"/>
     <mergeCell ref="AH3:AH4"/>
     <mergeCell ref="AI3:AI4"/>
     <mergeCell ref="AJ3:AJ4"/>
@@ -25409,12 +26420,6 @@
     <mergeCell ref="AE3:AE4"/>
     <mergeCell ref="AF3:AF4"/>
     <mergeCell ref="AG3:AG4"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="G1:N1"/>
-    <mergeCell ref="O1:P2"/>
-    <mergeCell ref="Q1:S2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="AC5:AC19">
     <cfRule type="cellIs" dxfId="23" priority="3" operator="lessThan">
@@ -25437,78 +26442,78 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -25598,10 +26603,10 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
     </row>
@@ -25693,8 +26698,8 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -27118,6 +28123,48 @@
         <v>0.32</v>
       </c>
       <c r="AE19" s="1">
+        <v>0.62422526589639604</v>
+      </c>
+    </row>
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AA21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB21">
+        <f>MIN(AB5:AB19)</f>
+        <v>12.632999999999999</v>
+      </c>
+      <c r="AC21">
+        <f>MIN(AC5:AC19)</f>
+        <v>17549</v>
+      </c>
+      <c r="AD21">
+        <f>MIN(AD5:AD19)</f>
+        <v>0.32</v>
+      </c>
+      <c r="AE21">
+        <f>MIN(AE5:AE19)</f>
+        <v>0.51863187696074597</v>
+      </c>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AA22" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <f>MAX(AB5:AB19)</f>
+        <v>18.088000000000001</v>
+      </c>
+      <c r="AC22">
+        <f>MAX(AC5:AC19)</f>
+        <v>17883</v>
+      </c>
+      <c r="AD22">
+        <f>MAX(AD5:AD19)</f>
+        <v>0.48</v>
+      </c>
+      <c r="AE22">
+        <f>MAX(AE5:AE19)</f>
         <v>0.62422526589639604</v>
       </c>
     </row>
@@ -27141,78 +28188,78 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -27302,25 +28349,25 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="AF3" s="12" t="s">
+      <c r="AF3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AG3" s="13" t="s">
+      <c r="AG3" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="AH3" s="13" t="s">
+      <c r="AH3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="AI3" s="13" t="s">
+      <c r="AI3" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="AJ3" s="13" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>46</v>
       </c>
     </row>
@@ -27412,13 +28459,13 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-      <c r="AI4" s="13"/>
-      <c r="AJ4" s="13"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
+      <c r="AF4" s="16"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="12"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -29070,8 +30117,56 @@
         <v>16.309999999999999</v>
       </c>
     </row>
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB21">
+        <f>MIN(AB5:AB19)</f>
+        <v>12.941000000000001</v>
+      </c>
+      <c r="AC21">
+        <f>MIN(AC5:AC19)</f>
+        <v>14100</v>
+      </c>
+      <c r="AD21">
+        <f>MIN(AD5:AD19)</f>
+        <v>0.61</v>
+      </c>
+      <c r="AE21">
+        <f>MIN(AE5:AE19)</f>
+        <v>0.40056622541893</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA22" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <f>MAX(AB5:AB19)</f>
+        <v>16.279</v>
+      </c>
+      <c r="AC22">
+        <f>MAX(AC5:AC19)</f>
+        <v>15460</v>
+      </c>
+      <c r="AD22">
+        <f>MAX(AD5:AD19)</f>
+        <v>0.69</v>
+      </c>
+      <c r="AE22">
+        <f>MAX(AE5:AE19)</f>
+        <v>0.42306220827913299</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:N1"/>
+    <mergeCell ref="O1:P2"/>
+    <mergeCell ref="Q1:S2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="J2:N2"/>
     <mergeCell ref="AH3:AH4"/>
     <mergeCell ref="AI3:AI4"/>
     <mergeCell ref="AJ3:AJ4"/>
@@ -29081,12 +30176,6 @@
     <mergeCell ref="AE3:AE4"/>
     <mergeCell ref="AF3:AF4"/>
     <mergeCell ref="AG3:AG4"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="G1:N1"/>
-    <mergeCell ref="O1:P2"/>
-    <mergeCell ref="Q1:S2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="AC5:AC19">
     <cfRule type="cellIs" dxfId="20" priority="21" operator="lessThan">
@@ -29104,6 +30193,8 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -29113,74 +30204,74 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -29270,10 +30361,10 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
     </row>
@@ -29365,8 +30456,8 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -31052,78 +32143,78 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="13" t="s">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="16" t="s">
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
-      <c r="AE2" s="16"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -31213,10 +32304,10 @@
       <c r="AC3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="14" t="s">
+      <c r="AD3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="AE3" s="14" t="s">
+      <c r="AE3" s="13" t="s">
         <v>38</v>
       </c>
     </row>
@@ -31308,8 +32399,8 @@
       <c r="AC4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="AD4" s="15"/>
-      <c r="AE4" s="15"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -32959,6 +34050,48 @@
       </c>
       <c r="AJ19">
         <v>23.89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA22" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB22">
+        <f>MIN(AB5:AB19)</f>
+        <v>15.244999999999999</v>
+      </c>
+      <c r="AC22">
+        <f>MIN(AC5:AC19)</f>
+        <v>16155</v>
+      </c>
+      <c r="AD22">
+        <f>MIN(AD5:AD19)</f>
+        <v>0.32</v>
+      </c>
+      <c r="AE22">
+        <f>MIN(AE5:AE19)</f>
+        <v>0.51687198714515203</v>
+      </c>
+    </row>
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AA23" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <f>MAX(AB5:AB19)</f>
+        <v>17.855</v>
+      </c>
+      <c r="AC23">
+        <f>MAX(AC5:AC19)</f>
+        <v>18149</v>
+      </c>
+      <c r="AD23">
+        <f>MAX(AD5:AD19)</f>
+        <v>0.39</v>
+      </c>
+      <c r="AE23">
+        <f>MAX(AE5:AE19)</f>
+        <v>0.635626291223506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>